<commit_message>
Updated Nicknames with a few more requested identifiers.
</commit_message>
<xml_diff>
--- a/Spatial_PDAC_NG2022/Nicknames_Select_Samples.xlsx
+++ b/Spatial_PDAC_NG2022/Nicknames_Select_Samples.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rjayasin/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{431E217C-7837-4E44-A379-9A5210A4C5C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7426E60A-C384-8D43-B5D1-D2485A7518E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18060" yWindow="-21820" windowWidth="34500" windowHeight="21820" xr2:uid="{2346DC3F-184C-8A4E-9067-11D1EACA9240}"/>
+    <workbookView xWindow="58100" yWindow="-7480" windowWidth="30240" windowHeight="18880" xr2:uid="{2346DC3F-184C-8A4E-9067-11D1EACA9240}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="56">
   <si>
     <t>HT190P1-S1H7A2K1G1Z1_1Bc1_1</t>
   </si>
@@ -144,19 +144,85 @@
   </si>
   <si>
     <t>Identifier</t>
+  </si>
+  <si>
+    <t>HT124P1-XB1_1</t>
+  </si>
+  <si>
+    <t>HT124P1-S1H1A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT124P1-S1H2A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT124P1-S1H4A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT124P1-XB2_1</t>
+  </si>
+  <si>
+    <t>HT123P1-S1H1A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT123P1-S1H3A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT123P1-S1H5A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT124P1-XB3_1</t>
+  </si>
+  <si>
+    <t>HT125P1-S1H3A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT125P1-S1H4A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT125P1-S1H8A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT125P1-S1H9A2K1G1Z1B1</t>
+  </si>
+  <si>
+    <t>HT123P1-XB1_1</t>
+  </si>
+  <si>
+    <t>HT123P1-XB2_1</t>
+  </si>
+  <si>
+    <t>HT123P1-XB3_1</t>
+  </si>
+  <si>
+    <t>HT125P1-XB1_1</t>
+  </si>
+  <si>
+    <t>HT125P1-XB2_1</t>
+  </si>
+  <si>
+    <t>HT125P1-XB3_1</t>
+  </si>
+  <si>
+    <t>HT125P1-XB4_1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -179,8 +245,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -515,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2204D90C-0C67-4E49-9A35-5DB3524C1180}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.5" bestFit="1" customWidth="1"/>
@@ -809,6 +876,90 @@
         <v>33</v>
       </c>
     </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>